<commit_message>
WIP checkpoint (auto, every 15 min): Parts 2/3 edits in progress, not yet checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4hHp37cV1PSzEtykqYjK1
</commit_message>
<xml_diff>
--- a/Data Science/Analyst-to-Architect/companion/ch10/ch10_practice.xlsx
+++ b/Data Science/Analyst-to-Architect/companion/ch10/ch10_practice.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cell detective" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Customers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Products" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Targets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cell detective" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12971,7 +12971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -13056,6 +13056,18 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>a code stored as text, so it keeps its zeros</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>